<commit_message>
Grid artworks with page for each artwork
</commit_message>
<xml_diff>
--- a/artwork_indexing/artworkPlaceholder.xlsx
+++ b/artwork_indexing/artworkPlaceholder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\becky\iCloudDrive\Documents\website_stuff\websites2026\bonnie\notes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oxuser\Desktop\Research\websites\the_website_files_themselves\bonnie\artwork_indexing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12E35C1-B8E2-478A-B877-00455EC4D3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3877BD92-5114-4088-A668-04729DDE3EC6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Artworks" sheetId="1" r:id="rId1"/>
@@ -145,9 +145,6 @@
     <t>forest.jpg</t>
   </si>
   <si>
-    <t xml:space="preserve">There was a time that I was so stressed that all I could do was watch this video on my projector. I made myself believe that it was my window because I lived in faerieland and did not go to university nor took exams. Instead I had other problems, better problems, like curses. </t>
-  </si>
-  <si>
     <t>faerie, curses</t>
   </si>
   <si>
@@ -164,6 +161,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://drive.google.com/drive/folders/1SzbpqiwrxSyGzQwjqXpgU0ej4n4gcvLj?usp=drive_link </t>
+  </si>
+  <si>
+    <t>There was a time that I was so stressed that all I could do was watch this video on my projector. I made myself believe that it was my window because I lived in faerieland and did not go to university nor took exams.</t>
   </si>
 </sst>
 </file>
@@ -627,14 +627,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.76953125" customWidth="1"/>
+    <col min="1" max="1" width="25.77734375" customWidth="1"/>
     <col min="2" max="7" width="26" style="15" customWidth="1"/>
     <col min="8" max="10" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="4" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:10" s="4" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -666,7 +666,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="9" customFormat="1" ht="22.1" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:10" s="9" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
@@ -674,10 +674,10 @@
         <v>32</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="11"/>
@@ -686,18 +686,18 @@
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
     </row>
-    <row r="3" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B3" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>47</v>
-      </c>
       <c r="D3" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
@@ -706,7 +706,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -726,7 +726,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" ht="22.1" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -746,7 +746,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" ht="24.65" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:10" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -757,7 +757,7 @@
         <v>31</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
@@ -766,7 +766,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" ht="22.1" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -786,7 +786,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10" ht="25.85" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:10" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -800,7 +800,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -814,7 +814,7 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="30.65" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:10" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
@@ -834,7 +834,7 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="22.1" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -850,7 +850,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -864,7 +864,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10" ht="26.4" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:10" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>21</v>
       </c>
@@ -880,7 +880,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10" ht="31.2" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:10" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>19</v>
       </c>
@@ -891,7 +891,7 @@
         <v>38</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
@@ -900,7 +900,7 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" ht="31.2" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:10" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>24</v>
       </c>
@@ -914,7 +914,7 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10" ht="26.4" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:10" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -928,7 +928,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:1" ht="111.65" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:1" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
     </row>
   </sheetData>

</xml_diff>